<commit_message>
Capgemini HTD Vtiger Automation Project
</commit_message>
<xml_diff>
--- a/CRM.BITM.Vtiger/src/test/resources/TestData.xlsx
+++ b/CRM.BITM.Vtiger/src/test/resources/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\git\vtigerRepo\CRM.BITM.Vtiger\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FD69F1-0B28-4E95-BCDA-A865F84D880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C54726-2607-4350-AABE-89DDE2EC5570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB9567A7-4C8E-46EA-B7A3-EA2DB94F2E41}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{CB9567A7-4C8E-46EA-B7A3-EA2DB94F2E41}"/>
   </bookViews>
   <sheets>
     <sheet name="VendorData" sheetId="1" r:id="rId1"/>
@@ -205,7 +205,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,6 +234,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -252,10 +260,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -284,8 +293,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -665,7 +678,7 @@
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="12" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="7">
@@ -707,7 +720,7 @@
       <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="12" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="7">
@@ -749,7 +762,7 @@
       <c r="A4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="7">
@@ -788,6 +801,11 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{B1ABB738-AF15-48E6-9631-D9C40AC78853}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{8CE147D1-51A1-4D8A-9D57-8EF736808F5E}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{908250DE-A5F0-4FF2-9D06-35EA6F4CAF9D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>